<commit_message>
feat: insights mock, templates XLSX, migrations ingestão/geo e docs
- Ingestão: colunas vendas (NF, hierarquia, unidade), templates em public/
- Migrations 004–007 (itens.unidade, codigo_externo vendedores, geo clientes, insights)
- Rota /insights com abas Território/Clientes e dados mock
- Documentação de contrato e dívida técnica de normatização

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/templates/template_relatorios_completo.xlsx
+++ b/docs/templates/template_relatorios_completo.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:P4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -411,6 +411,11 @@
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
     <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,34 +423,49 @@
         <v>data_venda</v>
       </c>
       <c r="B1" t="str">
+        <v>numero_nf</v>
+      </c>
+      <c r="C1" t="str">
         <v>cnpj_cliente</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>nome_cliente</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>codigo_vendedor</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>nome_vendedor</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>codigo_supervisor</v>
+      </c>
+      <c r="H1" t="str">
+        <v>nome_supervisor</v>
+      </c>
+      <c r="I1" t="str">
+        <v>codigo_gerente</v>
+      </c>
+      <c r="J1" t="str">
+        <v>nome_gerente</v>
+      </c>
+      <c r="K1" t="str">
         <v>sku</v>
       </c>
-      <c r="G1" t="str">
+      <c r="L1" t="str">
         <v>descricao_produto</v>
       </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
         <v>quantidade</v>
       </c>
-      <c r="I1" t="str">
+      <c r="N1" t="str">
+        <v>unidade</v>
+      </c>
+      <c r="O1" t="str">
         <v>valor_unitario</v>
       </c>
-      <c r="J1" t="str">
+      <c r="P1" t="str">
         <v>valor_total</v>
-      </c>
-      <c r="K1" t="str">
-        <v>codigo_supervisor</v>
       </c>
     </row>
     <row r="2">
@@ -453,34 +473,49 @@
         <v>12/03/2026</v>
       </c>
       <c r="B2" t="str">
+        <v>123456</v>
+      </c>
+      <c r="C2" t="str">
         <v>12345678000199</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Mercado Exemplo</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>V001</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>João Silva</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
+        <v>S001</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Pedro Costa</v>
+      </c>
+      <c r="I2" t="str">
+        <v>G001</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Maria Gerência</v>
+      </c>
+      <c r="K2" t="str">
         <v>CAMP-001</v>
       </c>
-      <c r="G2" t="str">
+      <c r="L2" t="str">
         <v>Produto Campestre 1kg</v>
       </c>
-      <c r="H2">
+      <c r="M2">
         <v>10</v>
       </c>
-      <c r="I2">
+      <c r="N2" t="str">
+        <v>UN</v>
+      </c>
+      <c r="O2">
         <v>25.9</v>
       </c>
-      <c r="J2">
+      <c r="P2">
         <v>259</v>
-      </c>
-      <c r="K2" t="str">
-        <v>S001</v>
       </c>
     </row>
     <row r="3">
@@ -488,39 +523,104 @@
         <v>12/03/2026</v>
       </c>
       <c r="B3" t="str">
+        <v>123456</v>
+      </c>
+      <c r="C3" t="str">
+        <v>12345678000199</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Mercado Exemplo</v>
+      </c>
+      <c r="E3" t="str">
+        <v>V001</v>
+      </c>
+      <c r="F3" t="str">
+        <v>João Silva</v>
+      </c>
+      <c r="G3" t="str">
+        <v>S001</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pedro Costa</v>
+      </c>
+      <c r="I3" t="str">
+        <v>G001</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Maria Gerência</v>
+      </c>
+      <c r="K3" t="str">
+        <v>CAMP-002</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Produto Campestre 500g</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+      <c r="N3" t="str">
+        <v>UN</v>
+      </c>
+      <c r="O3">
+        <v>14.5</v>
+      </c>
+      <c r="P3">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>12/03/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>123457</v>
+      </c>
+      <c r="C4" t="str">
         <v>98765432000188</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D4" t="str">
         <v>Supermercado Teste</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E4" t="str">
         <v>V001</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F4" t="str">
         <v>João Silva</v>
       </c>
-      <c r="F3" t="str">
-        <v>CAMP-002</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Produto Campestre 500g</v>
-      </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="I3">
-        <v>14.5</v>
-      </c>
-      <c r="J3">
-        <v>72.5</v>
-      </c>
-      <c r="K3" t="str">
+      <c r="G4" t="str">
         <v>S001</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Pedro Costa</v>
+      </c>
+      <c r="I4" t="str">
+        <v>G001</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Maria Gerência</v>
+      </c>
+      <c r="K4" t="str">
+        <v>CAMP-001</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Produto Campestre 1kg</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4" t="str">
+        <v>CX</v>
+      </c>
+      <c r="O4">
+        <v>25.9</v>
+      </c>
+      <c r="P4">
+        <v>51.8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>